<commit_message>
엑셀 자동 동기화: files/diet-reference-config-v1.0.0.xlsx
</commit_message>
<xml_diff>
--- a/files/diet-reference-config-v1.0.0.xlsx
+++ b/files/diet-reference-config-v1.0.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\이사라\Documents\Project_maiReport\outputs\mai-report-policy\식이\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{768A1CE9-0F11-4F68-9366-4FC526DCD996}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67F63235-CDE0-478D-97DC-0C542F684407}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38290" yWindow="-810" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10173" uniqueCount="2897">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10183" uniqueCount="2897">
   <si>
     <t>시트</t>
   </si>
@@ -54220,8 +54220,12 @@
       <c r="N173" s="19" t="s">
         <v>1716</v>
       </c>
-      <c r="O173" s="9"/>
-      <c r="P173" s="9"/>
+      <c r="O173" s="17" t="s">
+        <v>1683</v>
+      </c>
+      <c r="P173" s="17" t="s">
+        <v>99</v>
+      </c>
       <c r="Q173" s="9"/>
     </row>
     <row r="174" spans="1:17" ht="26">
@@ -54265,8 +54269,12 @@
       <c r="N174" s="19" t="s">
         <v>1716</v>
       </c>
-      <c r="O174" s="9"/>
-      <c r="P174" s="9"/>
+      <c r="O174" s="17" t="s">
+        <v>1685</v>
+      </c>
+      <c r="P174" s="17" t="s">
+        <v>99</v>
+      </c>
       <c r="Q174" s="9"/>
     </row>
     <row r="175" spans="1:17">
@@ -54310,8 +54318,12 @@
       <c r="N175" s="19" t="s">
         <v>1716</v>
       </c>
-      <c r="O175" s="9"/>
-      <c r="P175" s="9"/>
+      <c r="O175" s="17" t="s">
+        <v>1686</v>
+      </c>
+      <c r="P175" s="17" t="s">
+        <v>99</v>
+      </c>
       <c r="Q175" s="9"/>
     </row>
     <row r="176" spans="1:17">
@@ -54353,8 +54365,12 @@
       <c r="N176" s="19" t="s">
         <v>1723</v>
       </c>
-      <c r="O176" s="9"/>
-      <c r="P176" s="9"/>
+      <c r="O176" s="17" t="s">
+        <v>1687</v>
+      </c>
+      <c r="P176" s="17" t="s">
+        <v>99</v>
+      </c>
       <c r="Q176" s="9"/>
     </row>
     <row r="177" spans="1:17">
@@ -54396,8 +54412,12 @@
       <c r="N177" s="19" t="s">
         <v>1723</v>
       </c>
-      <c r="O177" s="9"/>
-      <c r="P177" s="9"/>
+      <c r="O177" s="17" t="s">
+        <v>1688</v>
+      </c>
+      <c r="P177" s="17" t="s">
+        <v>99</v>
+      </c>
       <c r="Q177" s="9"/>
     </row>
     <row r="178" spans="1:17">

</xml_diff>